<commit_message>
Execution Completed Nov-27 and Fixed P1 Failed scripts
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P3/Cypress/fixtures/BankMasterTemplate.xlsx
+++ b/Encollect_Web_SCB_P3/Cypress/fixtures/BankMasterTemplate.xlsx
@@ -412,112 +412,112 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Gerhold LLC Bank</v>
+        <v>Beahan - Hayes Bank</v>
       </c>
       <c r="B2" t="str">
-        <v>Haroldburgh Branch</v>
+        <v>Haltom City Branch</v>
       </c>
       <c r="C2" t="str">
-        <v>NSEHBY</v>
+        <v>05A2MK</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Kirlin, Donnelly and Koss Bank</v>
+        <v>Becker and Sons Bank</v>
       </c>
       <c r="B3" t="str">
-        <v>New Juana Branch</v>
+        <v>New Josephinestad Branch</v>
       </c>
       <c r="C3" t="str">
-        <v>IDTLXL</v>
+        <v>OZ4XAK</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Johnston Inc Bank</v>
+        <v>Koepp, Halvorson and Terry Bank</v>
       </c>
       <c r="B4" t="str">
-        <v>West Annabell Branch</v>
+        <v>McLean Branch</v>
       </c>
       <c r="C4" t="str">
-        <v>C1SLES</v>
+        <v>KA9T2B</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Denesik LLC Bank</v>
+        <v>Wiegand Inc Bank</v>
       </c>
       <c r="B5" t="str">
-        <v>New Noemy Branch</v>
+        <v>Pompano Beach Branch</v>
       </c>
       <c r="C5" t="str">
-        <v>9LSYON</v>
+        <v>LLV1IU</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sawayn, Schultz and Grant Bank</v>
+        <v>Langworth - Krajcik Bank</v>
       </c>
       <c r="B6" t="str">
-        <v>New Jack Branch</v>
+        <v>Turnerfurt Branch</v>
       </c>
       <c r="C6" t="str">
-        <v>VZERJF</v>
+        <v>ARMUWC</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Lehner - Dickinson Bank</v>
+        <v>Tremblay - Willms Bank</v>
       </c>
       <c r="B7" t="str">
-        <v>Breitenbergview Branch</v>
+        <v>Handton Branch</v>
       </c>
       <c r="C7" t="str">
-        <v>ZI1SJY</v>
+        <v>EQBRFE</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Macejkovic - Herman Bank</v>
+        <v>Stark, Fisher and Marquardt Bank</v>
       </c>
       <c r="B8" t="str">
-        <v>New Sonnytown Branch</v>
+        <v>North Newellshire Branch</v>
       </c>
       <c r="C8" t="str">
-        <v>RUHGZO</v>
+        <v>M2B5RV</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Ratke Group Bank</v>
+        <v>Gibson - Carter Bank</v>
       </c>
       <c r="B9" t="str">
-        <v>New Haven Branch</v>
+        <v>New Cortez Branch</v>
       </c>
       <c r="C9" t="str">
-        <v>HGIES9</v>
+        <v>YUI5TU</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Ruecker - Luettgen Bank</v>
+        <v>Windler - Wisozk Bank</v>
       </c>
       <c r="B10" t="str">
-        <v>East Nilstown Branch</v>
+        <v>Port Bailey Branch</v>
       </c>
       <c r="C10" t="str">
-        <v>JTYAVS</v>
+        <v>NJIF4C</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Roberts, Stark and Lebsack Bank</v>
+        <v>Tremblay, Harber and West Bank</v>
       </c>
       <c r="B11" t="str">
-        <v>Fort Joshua Branch</v>
+        <v>Port Lionel Branch</v>
       </c>
       <c r="C11" t="str">
-        <v>OW6VIN</v>
+        <v>TE04ES</v>
       </c>
     </row>
   </sheetData>

</xml_diff>